<commit_message>
add 8B R8 and 70B R8
</commit_message>
<xml_diff>
--- a/advanced-prompting/csv/merged_answers_new30.xlsx
+++ b/advanced-prompting/csv/merged_answers_new30.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,60 +521,70 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>llama_8B_R8</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>llama3.1-8B R16</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>llama3.1-8B R32</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Llama3.1-70B base</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Llama3.1-70B FT-50</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Llama3.1-70B FT-100</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Llama3.1-70B FT-150</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Llama3.1-70B FT-200</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Llama3.1-70B FT</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Llama3.1-70B QSP</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Llama3.1-70B FT+QSP</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>llama_70B_R8</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>llama3.1-70B R16</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>llama3.1-70B R32</t>
         </is>

</xml_diff>